<commit_message>
feat: trigo, simulador na porteira e CI no GitHub Actions
- trigo (Wheat, US HRW) no pipeline Parquet, nas conversões, na correlação de
  retornos, na correlação deslizante, na volatilidade e nas bandas de Bollinger;
  quebra de definição de jul/2020 marcada; defasagem e backtest seguem só com
  soja e milho (incluir o trigo mudaria os p-valores ajustados)
- simulador de stress cambial "na porteira": prêmio de porto e frete interno;
  R$/t = (soja US$/t + prêmio) x dólar - frete (preco_na_porteira), com
  premissas do usuário explicitadas e sem prometer o preço real recebido
- .github/workflows/pytest.yml: pytest em Ubuntu, Python 3.12, pip install -e ".[dev]"
- layout top-down: KPIs lado a lado e gráficos principais em largura total
- testes e fixtures atualizados para a terceira commodity; README atualizado

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/pink_sheet_amostra.xlsx
+++ b/tests/fixtures/pink_sheet_amostra.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE16"/>
+  <dimension ref="A1:AF16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -596,6 +596,11 @@
           <t>Maize</t>
         </is>
       </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Wheat, US HRW</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -748,6 +753,11 @@
           <t>($/mt)</t>
         </is>
       </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>($/mt)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -865,6 +875,9 @@
       <c r="AE7" t="n">
         <v>45</v>
       </c>
+      <c r="AF7" t="n">
+        <v>59.9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -962,6 +975,9 @@
       <c r="AE8" t="n">
         <v>167.3</v>
       </c>
+      <c r="AF8" t="n">
+        <v>201.2</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1059,6 +1075,9 @@
       <c r="AE9" t="n">
         <v>161.8</v>
       </c>
+      <c r="AF9" t="n">
+        <v>194</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1158,6 +1177,9 @@
       <c r="AE10" t="n">
         <v>198.8</v>
       </c>
+      <c r="AF10" t="n">
+        <v>268.6</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1257,6 +1279,9 @@
       <c r="AE11" t="n">
         <v>234.5</v>
       </c>
+      <c r="AF11" t="n">
+        <v>289.3</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1356,6 +1381,9 @@
       <c r="AE12" t="n">
         <v>202.6</v>
       </c>
+      <c r="AF12" t="n">
+        <v>252.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1455,6 +1483,9 @@
       <c r="AE13" t="n">
         <v>214.4</v>
       </c>
+      <c r="AF13" t="n">
+        <v>254.1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1554,6 +1585,9 @@
       <c r="AE14" t="n">
         <v>213.4</v>
       </c>
+      <c r="AF14" t="n">
+        <v>310</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1653,6 +1687,9 @@
       <c r="AE15" t="n">
         <v>224</v>
       </c>
+      <c r="AF15" t="n">
+        <v>330</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1751,6 +1788,9 @@
       </c>
       <c r="AE16" t="n">
         <v>239.6</v>
+      </c>
+      <c r="AF16" t="n">
+        <v>347</v>
       </c>
     </row>
   </sheetData>

</xml_diff>